<commit_message>
Rename LN-PCC and revamp result exports
Renames LN-PCC to PCC+GCN across plotting and table-generation scripts, updates labels/messages to English, and improves plotting robustness with safer save/error handling and modern colormap usage. Enhances table outputs by adding combined summary+rank views, aligning Excel/LaTeX conditional highlighting for gains and best ranks, and regenerates result artifacts (plots, TeX, and XLSX) with the new naming and formatting.
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -7,12 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="LN-PCC Absoluto" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Ganho vs GCN" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Resumo Médio" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Ranking" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="HP por Dataset" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="HP por Cenário" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="PCC+GCN Absolute" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Gain vs GCN" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Average Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Summary + Rank" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Ranking" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="HP by Dataset" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="HP by Scenario" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -47,7 +48,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -66,22 +67,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00A8D08D"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFD700"/>
       </patternFill>
     </fill>
     <fill>
@@ -193,13 +189,13 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -586,14 +582,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>LN-PCC Acurácia Absoluta (%)</t>
+          <t>PCC+GCN Absolute Accuracy (%)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ruído</t>
+          <t>Noise</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -1242,7 +1238,7 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Média</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="B19" s="6" t="n">
@@ -1309,14 +1305,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Ganho de LN-PCC vs GCN (pp)</t>
+          <t>PCC+GCN Gain vs GCN (pp)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ruído</t>
+          <t>Noise</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -1965,7 +1961,7 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Média</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="B19" s="10" t="n">
@@ -2022,14 +2018,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Acurácia Média (Todos os cenários)</t>
+          <t>Average Accuracy (All Scenarios)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Método</t>
+          <t>Method</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -2084,7 +2080,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Média</t>
+          <t>Average</t>
         </is>
       </c>
     </row>
@@ -2529,7 +2525,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>LN-PCC</t>
+          <t>PCC+GCN</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
@@ -2572,6 +2568,611 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Average Accuracy and Average Rank by Method</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Cora</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>CiteSeer</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>PubMed</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Amazon-C</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Amazon-P</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>DBLP</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>BlogCatalog</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Flickr</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Amz-Rat.</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Roman-Emp.</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Average Rank</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>GCN</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>67.62</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>54.523125</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>63.96</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>73.423125</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>79.77500000000001</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>65.39125</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>64.22437499999999</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>48.183125</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>37.50375</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>31.36125</v>
+      </c>
+      <c r="L3" s="4" t="n">
+        <v>58.59650000000001</v>
+      </c>
+      <c r="M3" s="4" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>CGNN</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>66.36562499999999</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>51.14875</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>56.36</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>43.74</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>47.191875</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>58.50875</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>24.151875</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>11.765</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>34.0875</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>18.829375</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>41.214875</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>10.9</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>CLNode</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>66.123125</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>53.875</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>62.65812500000001</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>74.701875</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>79.67125</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>63.765625</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>63.353125</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>46.636875</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>36.79375</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>30.669375</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>57.82481249999999</v>
+      </c>
+      <c r="M5" s="4" t="n">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>68.216875</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>54.994375</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>64.355625</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>72.938125</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>78.74375000000001</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>66.78874999999999</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>63.25</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>42.75375</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>37.619375</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>30.47125</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>58.0131875</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>4.7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>CR-GNN</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>67.871875</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>53.486875</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>64.8425</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>45.739375</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>36.09375</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>65.970625</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>59.479375</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>32.141875</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>35.103125</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>23.371875</v>
+      </c>
+      <c r="L7" s="4" t="n">
+        <v>48.410125</v>
+      </c>
+      <c r="M7" s="4" t="n">
+        <v>7.6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>DGNN</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>57.72</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>47.97</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>61.641875</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>49.564375</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>55.045625</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>62.8475</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>42.54625</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>17.1675</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>34.345</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>21.2425</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>45.0090625</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>10.3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>NRGNN</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>71.005</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>60.100625</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>60.05125</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>65.91187499999999</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>71.39624999999999</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>71.80875</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>70.095</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>41.018125</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>36.341875</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>45.364375</v>
+      </c>
+      <c r="L9" s="4" t="n">
+        <v>59.3093125</v>
+      </c>
+      <c r="M9" s="4" t="n">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>PIGNN</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>66.440625</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>57.53875</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>66.00875000000001</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>74.17874999999999</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>79.748125</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>69.15375</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>52.876875</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>47.77</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>37.220625</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>30.213125</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>58.1149375</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>RNCGLN</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>70.93187500000001</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>59.700625</v>
+      </c>
+      <c r="D11" s="4" t="n"/>
+      <c r="E11" s="4" t="n">
+        <v>61.584375</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>68.481875</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>63.278125</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>55.7575</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>24.079375</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>31.1675</v>
+      </c>
+      <c r="K11" s="8" t="n">
+        <v>47.94125</v>
+      </c>
+      <c r="L11" s="4" t="n">
+        <v>53.65805555555556</v>
+      </c>
+      <c r="M11" s="4" t="n">
+        <v>6.666666666666667</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>RTGNN</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>64.013125</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>50.716875</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>63.104375</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>62.06375</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>76.425625</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>61.704375</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>69.729375</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>39.08375</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>36.185</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>45.6575</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>56.868375</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>7.1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>UnionNET</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>68.456875</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>58.40875</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>63.785</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>33.47</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>29.29875</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>65.829375</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>49.6125</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>21.07125</v>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>35.324375</v>
+      </c>
+      <c r="K13" s="4" t="n">
+        <v>15.208125</v>
+      </c>
+      <c r="L13" s="4" t="n">
+        <v>44.04649999999999</v>
+      </c>
+      <c r="M13" s="4" t="n">
+        <v>8.4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>PCC+GCN</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>68.730625</v>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>60.465</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>64.035</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>69.81812499999999</v>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>80.454375</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>68.87309375</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>66.1988875</v>
+      </c>
+      <c r="I14" s="8" t="n">
+        <v>49.77148125</v>
+      </c>
+      <c r="J14" s="8" t="n">
+        <v>38.53821875</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>35.80884375</v>
+      </c>
+      <c r="L14" s="8" t="n">
+        <v>60.26936499999999</v>
+      </c>
+      <c r="M14" s="8" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2586,14 +3187,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Ranking por Dataset</t>
+          <t>Ranking by Dataset</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Método</t>
+          <t>Method</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -2648,7 +3249,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Rank Médio</t>
+          <t>Average Rank</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3694,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>LN-PCC</t>
+          <t>PCC+GCN</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
@@ -3135,7 +3736,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3160,14 +3761,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>HPO (cenário clean por dataset)</t>
+          <t>HPO (clean scenario by dataset)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Parâmetro</t>
+          <t>Parameter</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -3853,7 +4454,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3979,7 +4580,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Ruído</t>
+          <t>Noise</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add average gain column and unify highlighting
The gain pipeline now computes a per-row `GLOBAL_MEAN` across datasets and includes it in terminal output, LaTeX, and Excel gain tables (labeled as `Average`). Gain styling was also simplified to a single threshold scheme: light green for > 0.5, light red for < -0.5, and no bold/strong-green tier. Regenerated `results.tex` and `results.xlsx` reflect the new column and formatting.
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -1286,7 +1286,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1300,6 +1300,7 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1365,6 +1366,11 @@
           <t>Roman-Emp.</t>
         </is>
       </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1402,6 +1408,9 @@
       <c r="K3" s="8" t="n">
         <v>5.66</v>
       </c>
+      <c r="L3" s="7" t="n">
+        <v>1.13</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1439,6 +1448,9 @@
       <c r="K4" s="8" t="n">
         <v>5.78</v>
       </c>
+      <c r="L4" s="7" t="n">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1476,6 +1488,9 @@
       <c r="K5" s="8" t="n">
         <v>4.8</v>
       </c>
+      <c r="L5" s="7" t="n">
+        <v>1.53</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -1513,6 +1528,9 @@
       <c r="K6" s="8" t="n">
         <v>4.08</v>
       </c>
+      <c r="L6" s="7" t="n">
+        <v>1.24</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1550,6 +1568,9 @@
       <c r="K7" s="8" t="n">
         <v>2.84</v>
       </c>
+      <c r="L7" s="7" t="n">
+        <v>1.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1587,6 +1608,9 @@
       <c r="K8" s="8" t="n">
         <v>6.07</v>
       </c>
+      <c r="L8" s="7" t="n">
+        <v>1.76</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1624,6 +1648,9 @@
       <c r="K9" s="8" t="n">
         <v>5.51</v>
       </c>
+      <c r="L9" s="7" t="n">
+        <v>1.61</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1661,6 +1688,9 @@
       <c r="K10" s="8" t="n">
         <v>2.32</v>
       </c>
+      <c r="L10" s="7" t="n">
+        <v>1.32</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1698,6 +1728,9 @@
       <c r="K11" s="8" t="n">
         <v>5.77</v>
       </c>
+      <c r="L11" s="8" t="n">
+        <v>2.13</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1735,6 +1768,9 @@
       <c r="K12" s="8" t="n">
         <v>4.94</v>
       </c>
+      <c r="L12" s="7" t="n">
+        <v>1.96</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1772,6 +1808,9 @@
       <c r="K13" s="8" t="n">
         <v>3.35</v>
       </c>
+      <c r="L13" s="8" t="n">
+        <v>2.11</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1809,6 +1848,9 @@
       <c r="K14" s="8" t="n">
         <v>4.71</v>
       </c>
+      <c r="L14" s="7" t="n">
+        <v>1.84</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1846,6 +1888,9 @@
       <c r="K15" s="8" t="n">
         <v>4.89</v>
       </c>
+      <c r="L15" s="7" t="n">
+        <v>1.06</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1883,6 +1928,9 @@
       <c r="K16" s="8" t="n">
         <v>3.07</v>
       </c>
+      <c r="L16" s="8" t="n">
+        <v>2.01</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1920,6 +1968,9 @@
       <c r="K17" s="8" t="n">
         <v>4.27</v>
       </c>
+      <c r="L17" s="8" t="n">
+        <v>2.47</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1957,6 +2008,9 @@
       <c r="K18" s="8" t="n">
         <v>3.11</v>
       </c>
+      <c r="L18" s="7" t="n">
+        <v>1.91</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1994,10 +2048,13 @@
       <c r="K19" s="8" t="n">
         <v>4.45</v>
       </c>
+      <c r="L19" s="10" t="n">
+        <v>1.67</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Improve plot styling and add summary analysis scripts
- Increase font sizes, line widths, and DPI across all plot scripts for better readability
- Add `framealpha` to legends and bold axis labels/ticks throughout
- Differentiate PCC+GCN line weight from other priority methods in `generate_plots_instance.py`
- Add `add_summary_sheets_to_excel.py`: writes Instance Accuracy, Training Time, and summary-by-noise-rate sheets to results.xlsx
- Add `scratch_summary_tables.py`: prints the same summary tables to stdout for quick inspection
- Update all regenerated plot images and results.xlsx
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -14,6 +14,10 @@
     <sheet name="Ranking" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="HP by Dataset" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="HP by Scenario" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Instance Accuracy" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Instance Training Time" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Summary by Noise Rate (Acc)" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Summary by Noise Rate (Gain)" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -48,7 +52,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -83,6 +87,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002F5597"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -156,7 +165,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -196,6 +205,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1280,6 +1298,2999 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Global Mean Accuracy across 10 Datasets by Noise Rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Noise Type</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Clean (0.0)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Avg (0.1-0.5)</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Overall Avg</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>INSTANCE</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>GCN</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>69.18000000000001</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>66.95999999999999</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>65.45999999999999</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>62.6</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>58.23</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>61.01</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>62.37</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>INSTANCE</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>68.48999999999999</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>66.17</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>64.47</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>61.99</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>58.04</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>50.97</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>60.33</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>61.69</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>INSTANCE</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>NRGNN</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>67.40000000000001</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>67.98999999999999</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>66.65000000000001</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>62.97</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>52.98</v>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>62.26</v>
+      </c>
+      <c r="J5" s="8" t="n">
+        <v>63.12</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>INSTANCE</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>PIGNN</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>66.2</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>55.16</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>52.76</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>51.06</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>48.64</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>44.84</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>50.49</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>53.11</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>INSTANCE</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>PCC+GCN</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>70.31</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>67.56999999999999</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>65.89</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>63.77</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>58.77</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>51.72</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>61.54</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>UNIFORM</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>CGNN</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>48.19</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>46.44</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>44.99</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>42.87</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>38.56</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>35.54</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>41.68</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>42.77</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>UNIFORM</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>CLNode</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>68.65000000000001</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>66.33</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>63.27</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>60.52</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>56.32</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>51.04</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>59.5</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>61.02</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>UNIFORM</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>68.48999999999999</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>66.06999999999999</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>63.67</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>60.82</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>56.86</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>51.51</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>59.79</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>61.24</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>UNIFORM</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>CR-GNN</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>59.85</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>54.6</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>52.04</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>50.3</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>46.46</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>40.58</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>50.64</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>UNIFORM</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>DGNN</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>56.64</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>52.63</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>44.89</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>40.71</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>36.56</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>44.56</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>46.57</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>UNIFORM</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>GCN</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>69.18000000000001</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>67.02</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>64.44</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>61.39</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>57.15</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>51.74</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>60.35</v>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>61.82</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>UNIFORM</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NRGNN</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>67.40000000000001</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>66.2</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>64.70999999999999</v>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>62.62</v>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>59.29</v>
+      </c>
+      <c r="H14" s="8" t="n">
+        <v>55.36</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>61.64</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>62.6</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>UNIFORM</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>PCC+GCN</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="n">
+        <v>70.31</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>68.22</v>
+      </c>
+      <c r="E15" s="8" t="n">
+        <v>65.95999999999999</v>
+      </c>
+      <c r="F15" s="8" t="n">
+        <v>62.62</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>58.64</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="I15" s="8" t="n">
+        <v>61.79</v>
+      </c>
+      <c r="J15" s="8" t="n">
+        <v>63.21</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>UNIFORM</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>PIGNN</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>66.2</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>65.04000000000001</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>63.67</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>61.07</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>57</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>52.48</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>59.85</v>
+      </c>
+      <c r="J16" s="4" t="n">
+        <v>60.91</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>UNIFORM</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>RNCGLN</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>60.99</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>59.19</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>57.74</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>55.08</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>54.65</v>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>55.25</v>
+      </c>
+      <c r="J17" s="4" t="n">
+        <v>56.21</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>UNIFORM</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>RTGNN</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>63.06</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>60.91</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>61.34</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>60.9</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>57.94</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>54.28</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>59.07</v>
+      </c>
+      <c r="J18" s="4" t="n">
+        <v>59.74</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>UNIFORM</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>UnionNET</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>53.94</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>51.88</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>50.01</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>47.88</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>43.99</v>
+      </c>
+      <c r="H19" s="4" t="n">
+        <v>39.77</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="J19" s="4" t="n">
+        <v>47.91</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>PAIR</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>CGNN</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>48.19</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>46.32</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>43.92</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>40.63</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>35.41</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>28.89</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>39.04</v>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>40.56</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>PAIR</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>CLNode</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>68.65000000000001</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>65.69</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>61.91</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>56.62</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>47.62</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>36.23</v>
+      </c>
+      <c r="I21" s="4" t="n">
+        <v>53.61</v>
+      </c>
+      <c r="J21" s="4" t="n">
+        <v>56.12</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>PAIR</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>68.48999999999999</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>65.56999999999999</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>61.63</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>56.52</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>47.76</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>36.52</v>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>56.08</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>PAIR</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>CR-GNN</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>59.85</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>56.21</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>51.68</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>46.27</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>41.75</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>45.66</v>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>48.03</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>PAIR</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>DGNN</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>56.64</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>52.93</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>49.11</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>43.67</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>40.14</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>31.55</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>43.48</v>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>45.67</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>PAIR</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>GCN</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>69.18000000000001</v>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>66.43000000000001</v>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>62.6</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>56.98</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>47.98</v>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>36.72</v>
+      </c>
+      <c r="I25" s="4" t="n">
+        <v>54.14</v>
+      </c>
+      <c r="J25" s="4" t="n">
+        <v>56.65</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>PAIR</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>NRGNN</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>67.40000000000001</v>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>65.95</v>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>62.99</v>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>58.59</v>
+      </c>
+      <c r="G26" s="4" t="n">
+        <v>49.25</v>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>37.02</v>
+      </c>
+      <c r="I26" s="4" t="n">
+        <v>54.76</v>
+      </c>
+      <c r="J26" s="4" t="n">
+        <v>56.87</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>PAIR</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>PCC+GCN</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="n">
+        <v>70.31</v>
+      </c>
+      <c r="D27" s="8" t="n">
+        <v>68.04000000000001</v>
+      </c>
+      <c r="E27" s="8" t="n">
+        <v>63.92</v>
+      </c>
+      <c r="F27" s="8" t="n">
+        <v>59.11</v>
+      </c>
+      <c r="G27" s="8" t="n">
+        <v>49.94</v>
+      </c>
+      <c r="H27" s="8" t="n">
+        <v>38.82</v>
+      </c>
+      <c r="I27" s="8" t="n">
+        <v>55.97</v>
+      </c>
+      <c r="J27" s="8" t="n">
+        <v>58.36</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>PAIR</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>PIGNN</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>66.2</v>
+      </c>
+      <c r="D28" s="4" t="n">
+        <v>64.84</v>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>61.66</v>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>57.26</v>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>48.86</v>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>36.62</v>
+      </c>
+      <c r="I28" s="4" t="n">
+        <v>53.85</v>
+      </c>
+      <c r="J28" s="4" t="n">
+        <v>55.91</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>PAIR</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>RNCGLN</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="n">
+        <v>60.99</v>
+      </c>
+      <c r="D29" s="4" t="n">
+        <v>58.87</v>
+      </c>
+      <c r="E29" s="4" t="n">
+        <v>57.04</v>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>50.99</v>
+      </c>
+      <c r="G29" s="4" t="n">
+        <v>42.79</v>
+      </c>
+      <c r="H29" s="4" t="n">
+        <v>33.79</v>
+      </c>
+      <c r="I29" s="4" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="J29" s="4" t="n">
+        <v>50.74</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>PAIR</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>RTGNN</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>63.06</v>
+      </c>
+      <c r="D30" s="4" t="n">
+        <v>62.14</v>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>54.92</v>
+      </c>
+      <c r="G30" s="4" t="n">
+        <v>46.61</v>
+      </c>
+      <c r="H30" s="4" t="n">
+        <v>36.53</v>
+      </c>
+      <c r="I30" s="4" t="n">
+        <v>51.98</v>
+      </c>
+      <c r="J30" s="4" t="n">
+        <v>53.83</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>PAIR</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>UnionNET</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="n">
+        <v>53.94</v>
+      </c>
+      <c r="D31" s="4" t="n">
+        <v>51.11</v>
+      </c>
+      <c r="E31" s="4" t="n">
+        <v>48.83</v>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>44.69</v>
+      </c>
+      <c r="G31" s="4" t="n">
+        <v>37.52</v>
+      </c>
+      <c r="H31" s="4" t="n">
+        <v>30.28</v>
+      </c>
+      <c r="I31" s="4" t="n">
+        <v>42.48</v>
+      </c>
+      <c r="J31" s="4" t="n">
+        <v>44.39</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>RANDOM</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>CGNN</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>48.19</v>
+      </c>
+      <c r="D32" s="4" t="n">
+        <v>47.12</v>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>46.01</v>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>42.49</v>
+      </c>
+      <c r="G32" s="4" t="n">
+        <v>38.68</v>
+      </c>
+      <c r="H32" s="4" t="n">
+        <v>33.38</v>
+      </c>
+      <c r="I32" s="4" t="n">
+        <v>41.53</v>
+      </c>
+      <c r="J32" s="4" t="n">
+        <v>42.64</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>RANDOM</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>CLNode</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="n">
+        <v>68.65000000000001</v>
+      </c>
+      <c r="D33" s="4" t="n">
+        <v>65.79000000000001</v>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>58.86</v>
+      </c>
+      <c r="G33" s="4" t="n">
+        <v>54.8</v>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>47.94</v>
+      </c>
+      <c r="I33" s="4" t="n">
+        <v>58.2</v>
+      </c>
+      <c r="J33" s="4" t="n">
+        <v>59.94</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>RANDOM</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="n">
+        <v>68.48999999999999</v>
+      </c>
+      <c r="D34" s="4" t="n">
+        <v>65.83</v>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>63.28</v>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>59.77</v>
+      </c>
+      <c r="G34" s="4" t="n">
+        <v>55.07</v>
+      </c>
+      <c r="H34" s="4" t="n">
+        <v>48.84</v>
+      </c>
+      <c r="I34" s="4" t="n">
+        <v>58.56</v>
+      </c>
+      <c r="J34" s="4" t="n">
+        <v>60.21</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>RANDOM</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>CR-GNN</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="n">
+        <v>59.85</v>
+      </c>
+      <c r="D35" s="4" t="n">
+        <v>55.95</v>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>53.32</v>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>49.21</v>
+      </c>
+      <c r="G35" s="4" t="n">
+        <v>45.13</v>
+      </c>
+      <c r="H35" s="4" t="n">
+        <v>38.82</v>
+      </c>
+      <c r="I35" s="4" t="n">
+        <v>48.48</v>
+      </c>
+      <c r="J35" s="4" t="n">
+        <v>50.38</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>RANDOM</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>DGNN</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="n">
+        <v>56.64</v>
+      </c>
+      <c r="D36" s="4" t="n">
+        <v>52.58</v>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>48.67</v>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>45.22</v>
+      </c>
+      <c r="G36" s="4" t="n">
+        <v>40.38</v>
+      </c>
+      <c r="H36" s="4" t="n">
+        <v>36.45</v>
+      </c>
+      <c r="I36" s="4" t="n">
+        <v>44.66</v>
+      </c>
+      <c r="J36" s="4" t="n">
+        <v>46.66</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>RANDOM</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>GCN</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="n">
+        <v>69.18000000000001</v>
+      </c>
+      <c r="D37" s="4" t="n">
+        <v>66.66</v>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>60.15</v>
+      </c>
+      <c r="G37" s="4" t="n">
+        <v>55.57</v>
+      </c>
+      <c r="H37" s="4" t="n">
+        <v>49.15</v>
+      </c>
+      <c r="I37" s="4" t="n">
+        <v>59.19</v>
+      </c>
+      <c r="J37" s="4" t="n">
+        <v>60.85</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>RANDOM</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>NRGNN</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="n">
+        <v>67.40000000000001</v>
+      </c>
+      <c r="D38" s="4" t="n">
+        <v>65.20999999999999</v>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>64.43000000000001</v>
+      </c>
+      <c r="F38" s="4" t="n">
+        <v>61.24</v>
+      </c>
+      <c r="G38" s="4" t="n">
+        <v>57.32</v>
+      </c>
+      <c r="H38" s="8" t="n">
+        <v>51.36</v>
+      </c>
+      <c r="I38" s="4" t="n">
+        <v>59.91</v>
+      </c>
+      <c r="J38" s="4" t="n">
+        <v>61.16</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>RANDOM</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>PCC+GCN</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="n">
+        <v>70.31</v>
+      </c>
+      <c r="D39" s="8" t="n">
+        <v>68.48999999999999</v>
+      </c>
+      <c r="E39" s="8" t="n">
+        <v>65.47</v>
+      </c>
+      <c r="F39" s="8" t="n">
+        <v>62.16</v>
+      </c>
+      <c r="G39" s="8" t="n">
+        <v>58.04</v>
+      </c>
+      <c r="H39" s="4" t="n">
+        <v>51.06</v>
+      </c>
+      <c r="I39" s="8" t="n">
+        <v>61.04</v>
+      </c>
+      <c r="J39" s="8" t="n">
+        <v>62.59</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>RANDOM</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>PIGNN</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="n">
+        <v>66.2</v>
+      </c>
+      <c r="D40" s="4" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="E40" s="4" t="n">
+        <v>63.21</v>
+      </c>
+      <c r="F40" s="4" t="n">
+        <v>59.91</v>
+      </c>
+      <c r="G40" s="4" t="n">
+        <v>56.71</v>
+      </c>
+      <c r="H40" s="4" t="n">
+        <v>50.49</v>
+      </c>
+      <c r="I40" s="4" t="n">
+        <v>59.02</v>
+      </c>
+      <c r="J40" s="4" t="n">
+        <v>60.22</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>RANDOM</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>RNCGLN</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="n">
+        <v>60.99</v>
+      </c>
+      <c r="D41" s="4" t="n">
+        <v>59.79</v>
+      </c>
+      <c r="E41" s="4" t="n">
+        <v>58.69</v>
+      </c>
+      <c r="F41" s="4" t="n">
+        <v>55.98</v>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>54.46</v>
+      </c>
+      <c r="H41" s="4" t="n">
+        <v>48.87</v>
+      </c>
+      <c r="I41" s="4" t="n">
+        <v>55.56</v>
+      </c>
+      <c r="J41" s="4" t="n">
+        <v>56.46</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>RANDOM</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>RTGNN</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="n">
+        <v>63.06</v>
+      </c>
+      <c r="D42" s="4" t="n">
+        <v>62.11</v>
+      </c>
+      <c r="E42" s="4" t="n">
+        <v>62.03</v>
+      </c>
+      <c r="F42" s="4" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="G42" s="4" t="n">
+        <v>56.58</v>
+      </c>
+      <c r="H42" s="4" t="n">
+        <v>50.66</v>
+      </c>
+      <c r="I42" s="4" t="n">
+        <v>58.31</v>
+      </c>
+      <c r="J42" s="4" t="n">
+        <v>59.11</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>RANDOM</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>UnionNET</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="n">
+        <v>53.94</v>
+      </c>
+      <c r="D43" s="4" t="n">
+        <v>45.59</v>
+      </c>
+      <c r="E43" s="4" t="n">
+        <v>45.33</v>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>41.73</v>
+      </c>
+      <c r="G43" s="4" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="H43" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="I43" s="4" t="n">
+        <v>40.97</v>
+      </c>
+      <c r="J43" s="4" t="n">
+        <v>43.13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Global Mean Accuracy Delta vs GCN across 10 Datasets (percentage points)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Noise Type</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Clean (0.0)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Average Delta</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>INSTANCE</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>GCN</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>INSTANCE</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="n">
+        <v>-0.6899999999999999</v>
+      </c>
+      <c r="D4" s="9" t="n">
+        <v>-0.79</v>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>-0.99</v>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>-0.62</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="H4" s="9" t="n">
+        <v>-0.83</v>
+      </c>
+      <c r="I4" s="9" t="n">
+        <v>-0.68</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>INSTANCE</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>NRGNN</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>-1.78</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>INSTANCE</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>PIGNN</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>-2.98</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>-11.8</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>-12.7</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>-11.55</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>-9.59</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>-6.96</v>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>-9.26</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>INSTANCE</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>PCC+GCN</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="F7" s="10" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="G7" s="10" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="I7" s="10" t="n">
+        <v>0.63</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>UNIFORM</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>CGNN</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>-20.99</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>-20.58</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>-19.45</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>-18.52</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>-18.6</v>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>-16.2</v>
+      </c>
+      <c r="I8" s="9" t="n">
+        <v>-19.05</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>UNIFORM</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>CLNode</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>-0.53</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>-0.6899999999999999</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>-1.17</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>-0.86</v>
+      </c>
+      <c r="G9" s="9" t="n">
+        <v>-0.83</v>
+      </c>
+      <c r="H9" s="9" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="I9" s="9" t="n">
+        <v>-0.8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>UNIFORM</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>-0.6899999999999999</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>-0.77</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>-0.5600000000000001</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>-0.29</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="I10" s="9" t="n">
+        <v>-0.58</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>UNIFORM</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>CR-GNN</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>-9.32</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>-12.42</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>-12.4</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>-11.09</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>-10.69</v>
+      </c>
+      <c r="H11" s="9" t="n">
+        <v>-11.16</v>
+      </c>
+      <c r="I11" s="9" t="n">
+        <v>-11.18</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>UNIFORM</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>DGNN</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>-12.53</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>-14.39</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>-16.43</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>-16.49</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>-16.44</v>
+      </c>
+      <c r="H12" s="9" t="n">
+        <v>-15.18</v>
+      </c>
+      <c r="I12" s="9" t="n">
+        <v>-15.24</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>UNIFORM</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>GCN</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>UNIFORM</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NRGNN</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>-1.78</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>-0.82</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>3.63</v>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>UNIFORM</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>PCC+GCN</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E15" s="10" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="F15" s="10" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="G15" s="10" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="I15" s="10" t="n">
+        <v>1.39</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>UNIFORM</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>PIGNN</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>-2.98</v>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>-1.98</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>-0.77</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>-0.32</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="I16" s="9" t="n">
+        <v>-0.91</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>UNIFORM</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>RNCGLN</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="n">
+        <v>-7.14</v>
+      </c>
+      <c r="D17" s="9" t="n">
+        <v>-6.98</v>
+      </c>
+      <c r="E17" s="9" t="n">
+        <v>-6.05</v>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>-5.73</v>
+      </c>
+      <c r="G17" s="9" t="n">
+        <v>-2.42</v>
+      </c>
+      <c r="H17" s="9" t="n">
+        <v>-2.03</v>
+      </c>
+      <c r="I17" s="9" t="n">
+        <v>-5.06</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>UNIFORM</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>RTGNN</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="n">
+        <v>-6.12</v>
+      </c>
+      <c r="D18" s="9" t="n">
+        <v>-6.11</v>
+      </c>
+      <c r="E18" s="9" t="n">
+        <v>-3.1</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>-0.49</v>
+      </c>
+      <c r="G18" s="7" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="H18" s="7" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="I18" s="9" t="n">
+        <v>-2.08</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>UNIFORM</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>UnionNET</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="n">
+        <v>-15.24</v>
+      </c>
+      <c r="D19" s="9" t="n">
+        <v>-15.14</v>
+      </c>
+      <c r="E19" s="9" t="n">
+        <v>-14.43</v>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>-13.51</v>
+      </c>
+      <c r="G19" s="9" t="n">
+        <v>-13.16</v>
+      </c>
+      <c r="H19" s="9" t="n">
+        <v>-11.97</v>
+      </c>
+      <c r="I19" s="9" t="n">
+        <v>-13.91</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>PAIR</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>CGNN</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="n">
+        <v>-20.99</v>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>-20.1</v>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>-18.68</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>-16.34</v>
+      </c>
+      <c r="G20" s="9" t="n">
+        <v>-12.57</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>-7.83</v>
+      </c>
+      <c r="I20" s="9" t="n">
+        <v>-16.09</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>PAIR</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>CLNode</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="n">
+        <v>-0.53</v>
+      </c>
+      <c r="D21" s="9" t="n">
+        <v>-0.74</v>
+      </c>
+      <c r="E21" s="9" t="n">
+        <v>-0.6899999999999999</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>-0.36</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>-0.36</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>-0.49</v>
+      </c>
+      <c r="I21" s="9" t="n">
+        <v>-0.53</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>PAIR</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="n">
+        <v>-0.6899999999999999</v>
+      </c>
+      <c r="D22" s="9" t="n">
+        <v>-0.86</v>
+      </c>
+      <c r="E22" s="9" t="n">
+        <v>-0.97</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>-0.46</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="I22" s="9" t="n">
+        <v>-0.57</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>PAIR</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>CR-GNN</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="n">
+        <v>-9.32</v>
+      </c>
+      <c r="D23" s="9" t="n">
+        <v>-10.22</v>
+      </c>
+      <c r="E23" s="9" t="n">
+        <v>-10.92</v>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>-10.71</v>
+      </c>
+      <c r="G23" s="9" t="n">
+        <v>-6.23</v>
+      </c>
+      <c r="H23" s="9" t="n">
+        <v>-4.32</v>
+      </c>
+      <c r="I23" s="9" t="n">
+        <v>-8.619999999999999</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>PAIR</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>DGNN</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="n">
+        <v>-12.53</v>
+      </c>
+      <c r="D24" s="9" t="n">
+        <v>-13.5</v>
+      </c>
+      <c r="E24" s="9" t="n">
+        <v>-13.49</v>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>-13.31</v>
+      </c>
+      <c r="G24" s="9" t="n">
+        <v>-7.84</v>
+      </c>
+      <c r="H24" s="9" t="n">
+        <v>-5.17</v>
+      </c>
+      <c r="I24" s="9" t="n">
+        <v>-10.97</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>PAIR</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>GCN</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>PAIR</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>NRGNN</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="n">
+        <v>-1.78</v>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="F26" s="7" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="G26" s="7" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I26" s="4" t="n">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>PAIR</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>PCC+GCN</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="D27" s="10" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="E27" s="10" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="F27" s="10" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="G27" s="10" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="H27" s="10" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="I27" s="10" t="n">
+        <v>1.71</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>PAIR</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>PIGNN</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="n">
+        <v>-2.98</v>
+      </c>
+      <c r="D28" s="9" t="n">
+        <v>-1.59</v>
+      </c>
+      <c r="E28" s="9" t="n">
+        <v>-0.9399999999999999</v>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="G28" s="7" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="I28" s="9" t="n">
+        <v>-0.74</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>PAIR</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>RNCGLN</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="n">
+        <v>-7.14</v>
+      </c>
+      <c r="D29" s="9" t="n">
+        <v>-6.66</v>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>-4.67</v>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>-5.33</v>
+      </c>
+      <c r="G29" s="9" t="n">
+        <v>-4.33</v>
+      </c>
+      <c r="H29" s="9" t="n">
+        <v>-2.23</v>
+      </c>
+      <c r="I29" s="9" t="n">
+        <v>-5.06</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>PAIR</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>RTGNN</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="n">
+        <v>-6.12</v>
+      </c>
+      <c r="D30" s="9" t="n">
+        <v>-4.29</v>
+      </c>
+      <c r="E30" s="9" t="n">
+        <v>-2.9</v>
+      </c>
+      <c r="F30" s="9" t="n">
+        <v>-2.06</v>
+      </c>
+      <c r="G30" s="9" t="n">
+        <v>-1.37</v>
+      </c>
+      <c r="H30" s="4" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="I30" s="9" t="n">
+        <v>-2.82</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>PAIR</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>UnionNET</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="n">
+        <v>-15.24</v>
+      </c>
+      <c r="D31" s="9" t="n">
+        <v>-15.32</v>
+      </c>
+      <c r="E31" s="9" t="n">
+        <v>-13.77</v>
+      </c>
+      <c r="F31" s="9" t="n">
+        <v>-12.29</v>
+      </c>
+      <c r="G31" s="9" t="n">
+        <v>-10.46</v>
+      </c>
+      <c r="H31" s="9" t="n">
+        <v>-6.44</v>
+      </c>
+      <c r="I31" s="9" t="n">
+        <v>-12.25</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>RANDOM</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>CGNN</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="n">
+        <v>-20.99</v>
+      </c>
+      <c r="D32" s="9" t="n">
+        <v>-19.54</v>
+      </c>
+      <c r="E32" s="9" t="n">
+        <v>-18.39</v>
+      </c>
+      <c r="F32" s="9" t="n">
+        <v>-17.66</v>
+      </c>
+      <c r="G32" s="9" t="n">
+        <v>-16.88</v>
+      </c>
+      <c r="H32" s="9" t="n">
+        <v>-15.77</v>
+      </c>
+      <c r="I32" s="9" t="n">
+        <v>-18.21</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>RANDOM</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>CLNode</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="n">
+        <v>-0.53</v>
+      </c>
+      <c r="D33" s="9" t="n">
+        <v>-0.87</v>
+      </c>
+      <c r="E33" s="9" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="F33" s="9" t="n">
+        <v>-1.29</v>
+      </c>
+      <c r="G33" s="9" t="n">
+        <v>-0.77</v>
+      </c>
+      <c r="H33" s="9" t="n">
+        <v>-1.21</v>
+      </c>
+      <c r="I33" s="9" t="n">
+        <v>-0.91</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>RANDOM</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="n">
+        <v>-0.6899999999999999</v>
+      </c>
+      <c r="D34" s="9" t="n">
+        <v>-0.83</v>
+      </c>
+      <c r="E34" s="9" t="n">
+        <v>-1.12</v>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>-0.38</v>
+      </c>
+      <c r="G34" s="4" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="H34" s="4" t="n">
+        <v>-0.31</v>
+      </c>
+      <c r="I34" s="9" t="n">
+        <v>-0.64</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>RANDOM</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>CR-GNN</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="n">
+        <v>-9.32</v>
+      </c>
+      <c r="D35" s="9" t="n">
+        <v>-10.71</v>
+      </c>
+      <c r="E35" s="9" t="n">
+        <v>-11.08</v>
+      </c>
+      <c r="F35" s="9" t="n">
+        <v>-10.94</v>
+      </c>
+      <c r="G35" s="9" t="n">
+        <v>-10.44</v>
+      </c>
+      <c r="H35" s="9" t="n">
+        <v>-10.34</v>
+      </c>
+      <c r="I35" s="9" t="n">
+        <v>-10.47</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>RANDOM</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>DGNN</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="n">
+        <v>-12.53</v>
+      </c>
+      <c r="D36" s="9" t="n">
+        <v>-14.08</v>
+      </c>
+      <c r="E36" s="9" t="n">
+        <v>-15.73</v>
+      </c>
+      <c r="F36" s="9" t="n">
+        <v>-14.92</v>
+      </c>
+      <c r="G36" s="9" t="n">
+        <v>-15.18</v>
+      </c>
+      <c r="H36" s="9" t="n">
+        <v>-12.7</v>
+      </c>
+      <c r="I36" s="9" t="n">
+        <v>-14.19</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>RANDOM</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>GCN</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>RANDOM</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>NRGNN</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="n">
+        <v>-1.78</v>
+      </c>
+      <c r="D38" s="9" t="n">
+        <v>-1.45</v>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F38" s="7" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G38" s="7" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="H38" s="7" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="I38" s="4" t="n">
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>RANDOM</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>PCC+GCN</t>
+        </is>
+      </c>
+      <c r="C39" s="10" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="D39" s="10" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="E39" s="10" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="F39" s="10" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="G39" s="10" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="H39" s="10" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="I39" s="10" t="n">
+        <v>1.74</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>RANDOM</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>PIGNN</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="n">
+        <v>-2.98</v>
+      </c>
+      <c r="D40" s="9" t="n">
+        <v>-1.86</v>
+      </c>
+      <c r="E40" s="9" t="n">
+        <v>-1.19</v>
+      </c>
+      <c r="F40" s="4" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="G40" s="7" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="H40" s="7" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="I40" s="9" t="n">
+        <v>-0.63</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>RANDOM</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>RNCGLN</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="n">
+        <v>-7.14</v>
+      </c>
+      <c r="D41" s="9" t="n">
+        <v>-6.07</v>
+      </c>
+      <c r="E41" s="9" t="n">
+        <v>-4.81</v>
+      </c>
+      <c r="F41" s="9" t="n">
+        <v>-3.46</v>
+      </c>
+      <c r="G41" s="9" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="H41" s="9" t="n">
+        <v>-0.61</v>
+      </c>
+      <c r="I41" s="9" t="n">
+        <v>-3.84</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>RANDOM</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>RTGNN</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="n">
+        <v>-6.12</v>
+      </c>
+      <c r="D42" s="9" t="n">
+        <v>-4.55</v>
+      </c>
+      <c r="E42" s="9" t="n">
+        <v>-2.37</v>
+      </c>
+      <c r="F42" s="4" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G42" s="7" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="H42" s="7" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="I42" s="9" t="n">
+        <v>-1.75</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>RANDOM</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>UnionNET</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="n">
+        <v>-15.24</v>
+      </c>
+      <c r="D43" s="9" t="n">
+        <v>-21.07</v>
+      </c>
+      <c r="E43" s="9" t="n">
+        <v>-19.07</v>
+      </c>
+      <c r="F43" s="9" t="n">
+        <v>-18.42</v>
+      </c>
+      <c r="G43" s="9" t="n">
+        <v>-17.36</v>
+      </c>
+      <c r="H43" s="9" t="n">
+        <v>-15.16</v>
+      </c>
+      <c r="I43" s="9" t="n">
+        <v>-17.72</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -14309,4 +17320,1039 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Mean Accuracy Comparison on Instance Noise (Rates 0.1 - 0.5 Average)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Cora</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>CiteSeer</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>PubMed</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>BlogCatalog</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Flickr</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>DBLP</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Amazon-C</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Amazon-P</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Amz-Rat.</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Roman-Emp.</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>GCN</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>70.98999999999999</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>59.46</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>65.25</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>65.75</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>49.43</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>71.77</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>75.70999999999999</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>81.34999999999999</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>37.54</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>32.87</v>
+      </c>
+      <c r="L3" s="4" t="n">
+        <v>61.01</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>70.42</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>60.01</v>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>66.08</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>64.73999999999999</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>46.47</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>72.17</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>73.73999999999999</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>80.98</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>37.55</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>31.14</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>60.33</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>NRGNN</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>72.3</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>62.87</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>73.08</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>55.3</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>75.02</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>67.73</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>78.02</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>37.06</v>
+      </c>
+      <c r="K5" s="8" t="n">
+        <v>36.23</v>
+      </c>
+      <c r="L5" s="8" t="n">
+        <v>62.26</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>PIGNN</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>72.73999999999999</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>64.73999999999999</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>40.02</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>57.75</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>48.23</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>60.54</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>27.94</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>80.58</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>37.01</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>15.36</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>50.49</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>PCC+GCN</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>70.97</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>60.37</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>65.18000000000001</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>66.36</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>49.99</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>71.48</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>76.5</v>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>81.83</v>
+      </c>
+      <c r="J7" s="8" t="n">
+        <v>37.62</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>35.13</v>
+      </c>
+      <c r="L7" s="4" t="n">
+        <v>61.54</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Training Time on Instance Noise (Stacked CPU, GPU, Total in seconds)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Cora</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>CiteSeer</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>PubMed</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>BlogCatalog</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Flickr</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>DBLP</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Amazon-C</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Amazon-P</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Amz-Rat.</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Roman-Emp.</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>GCN</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="L3" s="4" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="M3" s="4" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>GPU</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>4.07</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>4.17</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>5.06</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>3.41</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr"/>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C5" s="19" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="D5" s="19" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="E5" s="19" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="F5" s="19" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="G5" s="19" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="H5" s="19" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="I5" s="19" t="n">
+        <v>4.21</v>
+      </c>
+      <c r="J5" s="19" t="n">
+        <v>4.36</v>
+      </c>
+      <c r="K5" s="19" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="L5" s="19" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="M5" s="19" t="n">
+        <v>3.46</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>GPU</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>23.31</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>27.83</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>172.1</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>52.16</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>80.51000000000001</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>169.4</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>141.97</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>68.66</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>264.01</v>
+      </c>
+      <c r="L7" s="4" t="n">
+        <v>199</v>
+      </c>
+      <c r="M7" s="4" t="n">
+        <v>119.9</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr"/>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="n">
+        <v>23.32</v>
+      </c>
+      <c r="D8" s="19" t="n">
+        <v>27.85</v>
+      </c>
+      <c r="E8" s="19" t="n">
+        <v>172.14</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>52.21</v>
+      </c>
+      <c r="G8" s="19" t="n">
+        <v>80.59999999999999</v>
+      </c>
+      <c r="H8" s="19" t="n">
+        <v>169.46</v>
+      </c>
+      <c r="I8" s="19" t="n">
+        <v>142.01</v>
+      </c>
+      <c r="J8" s="19" t="n">
+        <v>68.68000000000001</v>
+      </c>
+      <c r="K8" s="19" t="n">
+        <v>264.06</v>
+      </c>
+      <c r="L8" s="19" t="n">
+        <v>199.05</v>
+      </c>
+      <c r="M8" s="19" t="n">
+        <v>119.94</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>NRGNN</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>2.89</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>14.37</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>51.69</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>16.43</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>13.37</v>
+      </c>
+      <c r="L9" s="4" t="n">
+        <v>11.75</v>
+      </c>
+      <c r="M9" s="4" t="n">
+        <v>13.24</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>GPU</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>21.03</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>27.47</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>142.12</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>43.35</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>58.43</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>156.62</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>119.74</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>54</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>229.09</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>186.86</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>103.87</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr"/>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="n">
+        <v>22.63</v>
+      </c>
+      <c r="D11" s="19" t="n">
+        <v>30.36</v>
+      </c>
+      <c r="E11" s="19" t="n">
+        <v>149.4</v>
+      </c>
+      <c r="F11" s="19" t="n">
+        <v>57.72</v>
+      </c>
+      <c r="G11" s="19" t="n">
+        <v>110.13</v>
+      </c>
+      <c r="H11" s="19" t="n">
+        <v>173.05</v>
+      </c>
+      <c r="I11" s="19" t="n">
+        <v>129.44</v>
+      </c>
+      <c r="J11" s="19" t="n">
+        <v>57.27</v>
+      </c>
+      <c r="K11" s="19" t="n">
+        <v>242.46</v>
+      </c>
+      <c r="L11" s="19" t="n">
+        <v>198.61</v>
+      </c>
+      <c r="M11" s="19" t="n">
+        <v>117.11</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>PIGNN</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>112.49</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>108.81</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>102.06</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>137.9</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>135.92</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>98.28</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>151.76</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>110.59</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>95.78</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>GPU</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>11.38</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>33.29</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>35.05</v>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="K13" s="4" t="n">
+        <v>40.59</v>
+      </c>
+      <c r="L13" s="4" t="n">
+        <v>37.49</v>
+      </c>
+      <c r="M13" s="4" t="n">
+        <v>30.4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="17" t="inlineStr"/>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="D14" s="19" t="n">
+        <v>13.92</v>
+      </c>
+      <c r="E14" s="19" t="n">
+        <v>147.09</v>
+      </c>
+      <c r="F14" s="19" t="n">
+        <v>140.61</v>
+      </c>
+      <c r="G14" s="19" t="n">
+        <v>135.35</v>
+      </c>
+      <c r="H14" s="19" t="n">
+        <v>174.3</v>
+      </c>
+      <c r="I14" s="19" t="n">
+        <v>170.96</v>
+      </c>
+      <c r="J14" s="19" t="n">
+        <v>127.78</v>
+      </c>
+      <c r="K14" s="19" t="n">
+        <v>192.35</v>
+      </c>
+      <c r="L14" s="19" t="n">
+        <v>148.08</v>
+      </c>
+      <c r="M14" s="19" t="n">
+        <v>126.18</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>PCC+GCN</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>8.029999999999999</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>11.72</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>25.68</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>27.81</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>85.56999999999999</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>33.11</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>44.68</v>
+      </c>
+      <c r="J15" s="4" t="n">
+        <v>17.94</v>
+      </c>
+      <c r="K15" s="4" t="n">
+        <v>43.96</v>
+      </c>
+      <c r="L15" s="4" t="n">
+        <v>210.22</v>
+      </c>
+      <c r="M15" s="4" t="n">
+        <v>50.87</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr"/>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>GPU</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>4.72</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>7.55</v>
+      </c>
+      <c r="J16" s="4" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="K16" s="4" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="M16" s="4" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr"/>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="n">
+        <v>10.04</v>
+      </c>
+      <c r="D17" s="19" t="n">
+        <v>13.85</v>
+      </c>
+      <c r="E17" s="19" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="F17" s="19" t="n">
+        <v>31.37</v>
+      </c>
+      <c r="G17" s="19" t="n">
+        <v>88.98</v>
+      </c>
+      <c r="H17" s="19" t="n">
+        <v>37.1</v>
+      </c>
+      <c r="I17" s="19" t="n">
+        <v>52.23</v>
+      </c>
+      <c r="J17" s="19" t="n">
+        <v>21.05</v>
+      </c>
+      <c r="K17" s="19" t="n">
+        <v>47.9</v>
+      </c>
+      <c r="L17" s="19" t="n">
+        <v>212.31</v>
+      </c>
+      <c r="M17" s="19" t="n">
+        <v>54.52</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Highlight best total time per dataset column
Track the row index of each method's 'Total' time row and highlight the minimum value per dataset column (excluding GCN) using the existing best_fill style.
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -17949,7 +17949,7 @@
       <c r="F8" s="19" t="n">
         <v>52.21</v>
       </c>
-      <c r="G8" s="19" t="n">
+      <c r="G8" s="8" t="n">
         <v>80.59999999999999</v>
       </c>
       <c r="H8" s="19" t="n">
@@ -18218,7 +18218,7 @@
       <c r="K14" s="19" t="n">
         <v>192.35</v>
       </c>
-      <c r="L14" s="19" t="n">
+      <c r="L14" s="8" t="n">
         <v>148.08</v>
       </c>
       <c r="M14" s="19" t="n">
@@ -18318,37 +18318,37 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="C17" s="19" t="n">
+      <c r="C17" s="8" t="n">
         <v>10.04</v>
       </c>
-      <c r="D17" s="19" t="n">
+      <c r="D17" s="8" t="n">
         <v>13.85</v>
       </c>
-      <c r="E17" s="19" t="n">
+      <c r="E17" s="8" t="n">
         <v>30.4</v>
       </c>
-      <c r="F17" s="19" t="n">
+      <c r="F17" s="8" t="n">
         <v>31.37</v>
       </c>
       <c r="G17" s="19" t="n">
         <v>88.98</v>
       </c>
-      <c r="H17" s="19" t="n">
+      <c r="H17" s="8" t="n">
         <v>37.1</v>
       </c>
-      <c r="I17" s="19" t="n">
+      <c r="I17" s="8" t="n">
         <v>52.23</v>
       </c>
-      <c r="J17" s="19" t="n">
+      <c r="J17" s="8" t="n">
         <v>21.05</v>
       </c>
-      <c r="K17" s="19" t="n">
+      <c r="K17" s="8" t="n">
         <v>47.9</v>
       </c>
       <c r="L17" s="19" t="n">
         <v>212.31</v>
       </c>
-      <c r="M17" s="19" t="n">
+      <c r="M17" s="8" t="n">
         <v>54.52</v>
       </c>
     </row>

</xml_diff>